<commit_message>
Complete Milestone 1 and 2 implementation
</commit_message>
<xml_diff>
--- a/Defect_Tracker Template_v0.1 (1).xlsx
+++ b/Defect_Tracker Template_v0.1 (1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOQ\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/03bb5f1981b8452f/Desktop/ai-resume-screening-engine/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA31996-50BE-48F6-88C6-1D354D407004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{3FA31996-50BE-48F6-88C6-1D354D407004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA372697-0DDB-47CD-8CF3-9FBD74FEEA00}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
   <si>
     <t>Sl No</t>
   </si>
@@ -102,6 +102,45 @@
   </si>
   <si>
     <t>Model response verified</t>
+  </si>
+  <si>
+    <t>Job role not found during tool execution</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Added exception handling for invalid job roles</t>
+  </si>
+  <si>
+    <t>Error message verified</t>
+  </si>
+  <si>
+    <t>Tool output was not initially integrated into workflow</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>Integrated Job Agent and job requirements into workflow</t>
+  </si>
+  <si>
+    <t>Complete workflow verified</t>
+  </si>
+  <si>
+    <t>Tool selection required request-based handling</t>
+  </si>
+  <si>
+    <t>Implemented rule-based Tool Selector</t>
+  </si>
+  <si>
+    <t>Tool selection verified</t>
   </si>
 </sst>
 </file>
@@ -212,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -229,10 +268,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -589,102 +631,180 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
+    <row r="2" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="10">
+        <v>46265</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="9" t="s">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="10">
+        <v>46268</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="9" t="s">
+      <c r="H3" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="9" t="s">
-        <v>24</v>
+      <c r="K3" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="10">
+        <v>46279</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" s="9" t="s">
+      <c r="G4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="8" t="s">
         <v>21</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+      <c r="K4" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="10">
+        <v>46282</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="10">
+        <v>46282</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
@@ -880,7 +1000,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1 G5:G1048576</xm:sqref>
+          <xm:sqref>G1 G7:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1057,18 +1177,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1090,18 +1210,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>